<commit_message>
corrigir typo nas datas
</commit_message>
<xml_diff>
--- a/data/condominio.xlsx
+++ b/data/condominio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedrohamacher\OneDrive\Documentos antigo\Projetos_jl\Streamlit\Dashboard Pelada\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="14_{AFBA81A4-2B23-449D-B209-30A32CB7CB1E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{B3428EA7-6856-4212-B670-CF3EDE330DD7}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="14_{AFBA81A4-2B23-449D-B209-30A32CB7CB1E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{C7BBF518-F9C7-45B2-B982-14E2EBDE0B1C}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19180" windowHeight="7870" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19180" windowHeight="7870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="notas" sheetId="1" r:id="rId1"/>
@@ -2986,7 +2986,7 @@
         <v>46190</v>
       </c>
       <c r="DA1" s="1">
-        <v>46569</v>
+        <v>46204</v>
       </c>
       <c r="DB1" s="1">
         <v>46211</v>

</xml_diff>